<commit_message>
fix(productos): segunda pasada de fixer sobre los 9 libros de Chocolatería (7 residuos del verificador independiente: columna del 40 % de materias añadidas, %% literal, mapas sin _notas, Title Case, freeze_panes, «Inmovilizado amortizable», nota_legal con artículo 183/201 y gate) + GUIA_BUILD_DIR en los generadores; regenerados tras el guion: gate_libros 9/9, verificar_guion 0 rotas, md5 build = dl; handoff §5-§6 con el cierre de la fase A2+B1 y el paso a paso de B2+C
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01339ov3ruQ44NhPJc9k4A6N
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/guia-chocolateria-obrador/calculadora-capex-chocolateria.xlsx
+++ b/astro-site/public/dl/guia-chocolateria-obrador/calculadora-capex-chocolateria.xlsx
@@ -287,7 +287,7 @@
   <commentList>
     <comment ref="A10" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 37/1992, de 28 de diciembre, del Impuesto sobre el Valor Añadido (BOE-A-1992-28740), texto consolidado · «Última modificación: 28 de febrero de 2026» (Art. 91.Dos.1.1.º (las siete letras: pan común, harinas panificables, leches, quesos, huevos, frutas/verduras/hortalizas/legumbres/tubérc...) · https://www.boe.es/buscar/act.php?id=BOE-A-1992-28740</t>
+        <t>Verificado el 12-09-2026 · Ley 37/1992, de 28 de diciembre, del Impuesto sobre el Valor Añadido (BOE-A-1992-28740), texto consolidado · «Última modificación: 28 de febrero de 2026» (Art. 91.Dos.1.1.º (las siete letras: pan común, harinas panificables, leches, qu...) · https://www.boe.es/buscar/act.php?id=BOE-A-1992-28740</t>
       </text>
     </comment>
     <comment ref="A20" authorId="0" shapeId="0">
@@ -297,7 +297,7 @@
     </comment>
     <comment ref="A21" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 7/2022, de 8 de abril, de residuos y suelos contaminados para una economía circular (BOE-A-2022-5809), texto consolidado · «Última modificación: 02 de abril de 2025» (Periodo de liquidación: trimestre natural, salvo IVA mensual (art. 82.1).) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
+        <t>Verificado el 12-09-2026 · Ley 7/2022, de 8 de abril, de residuos y suelos contaminados para una economía circular (BOE-A-2022-5809), texto consolidado · «Última modificación: 02 de abril de 2025» (Arts.) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
       </text>
     </comment>
   </commentList>
@@ -312,7 +312,7 @@
   <commentList>
     <comment ref="P18" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 7/2022 (BOE-A-2022-5809), arts. 68.1.a) y 73.d) (confirmada, con dos razones en vez de una: el art. 73.d) los deja no sujetos y, antes que eso, el ámbito objetivo del art. 68.1.a) son lo...) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
+        <t>Verificado el 12-09-2026 · Ley 7/2022 (BOE-A-2022-5809), arts. 68.1.a) y 73.d) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
       </text>
     </comment>
     <comment ref="P21" authorId="0" shapeId="0">
@@ -322,12 +322,12 @@
     </comment>
     <comment ref="P23" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Enumerados los 55 grupos del Anexo: 435, 439, 442, 452, 454, 474, 491, 495, 615, 641-647, 651-659, 662, 665, 691, 75... · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
+        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Enumerados los 55 grupos del Anexo: 435, 439, 442, 452, 454, 474, 491, 495, 615, 641-647, 651-659, 662, 665,...) · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
       </text>
     </comment>
     <comment ref="P26" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Dos límites del propio texto: queda fuera lo que tenga impacto en el patrimonio histórico-artístico o en el uso priv... · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
+        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Arts.) · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
       </text>
     </comment>
     <comment ref="P27" authorId="0" shapeId="0">
@@ -347,12 +347,12 @@
   <commentList>
     <comment ref="H8" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Reglamento (UE) 2023/1115 del Parlamento Europeo y del Consejo, de 31 de mayo de 2023 (EUDR) · texto consolidado CELEX:02023R1115-20251226 (versión 26-12-2025, 002.001) (El art. 3 exige tres condiciones acumulativas: libres de deforestación, producidos conforme a la legislación del país de produc... · https://eur-lex.europa.eu/legal-content/ES/TXT/HTML/?uri=CELEX:02023R1115-20251226</t>
+        <t>Verificado el 12-09-2026 · Reglamento (UE) 2023/1115 del Parlamento Europeo y del Consejo, de 31 de mayo de 2023 (EUDR) · texto consolidado CELEX:02023R1115-20251226 (versión 26-12-2025, 002.001) (Arts.) · https://eur-lex.europa.eu/legal-content/ES/TXT/HTML/?uri=CELEX:02023R1115-20251226</t>
       </text>
     </comment>
     <comment ref="H9" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Enumerados los 55 grupos del Anexo: 435, 439, 442, 452, 454, 474, 491, 495, 615, 641-647, 651-659, 662, 665, 691, 75... · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
+        <t>Verificado el 12-09-2026 · Ley 12/2012, de 26 de diciembre, de medidas urgentes de liberalización del comercio y de determinados servicios (BOE-A-2012-15595), texto consolidado · «Última modificación: 29... (Enumerados los 55 grupos del Anexo: 435, 439, 442, 452, 454, 474, 491, 495, 615, 641-647, 651-659, 662, 665,...) · https://www.boe.es/buscar/act.php?id=BOE-A-2012-15595</t>
       </text>
     </comment>
     <comment ref="H14" authorId="0" shapeId="0">
@@ -382,7 +382,7 @@
     </comment>
     <comment ref="A38" authorId="0" shapeId="0">
       <text>
-        <t>Verificado el 12-09-2026 · Ley 7/2022 (BOE-A-2022-5809), arts. 68.1.a) y 73.d) (confirmada, con dos razones en vez de una: el art. 73.d) los deja no sujetos y, antes que eso, el ámbito objetivo del art. 68.1.a) son lo...) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
+        <t>Verificado el 12-09-2026 · Ley 7/2022 (BOE-A-2022-5809), arts. 68.1.a) y 73.d) · https://www.boe.es/buscar/act.php?id=BOE-A-2022-5809</t>
       </text>
     </comment>
   </commentList>
@@ -6101,7 +6101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -6511,17 +6511,38 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24" ht="44" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Inmovilizado amortizable</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>'CAPEX por Bloque'!L44-'CAPEX por Bloque'!L36-'CAPEX por Bloque'!L24</f>
+        <v>83614.99</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CAPEX por Bloque</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>CAPEX sin el fondo de maniobra, menos la fianza (es un depósito: se recupera, no se amortiza) y menos «packaging y moldes» (son existencias, no inmovilizado). Es la base que el libro 7 trae en su celda verde: compárala con la suya para comprobar que los dos libros dicen lo mismo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Si alguna de estas cifras no te cuadra, no la cambies aquí: esta hoja no tiene ni una celda editable. Vuelve a la hoja donde nace y cambia el parámetro o el importe. Es lo que evita que un resumen y su origen digan cosas distintas.</t>
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26" ht="80" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="26"/>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>LAS DOS PRIMERAS LÍNEAS DE DINERO SON DOS Y NO UNA A PROPÓSITO. «CAPEX sin el fondo de maniobra» es lo que le llevas al libro 7 y lo que se parece a lo que el sector llama «inversión de apertura»; el fondo de maniobra es caja, no inversión, y lo dota el libro 7 con sus meses de colchón y sus gastos fijos. La suma de las dos es la inversión total, y sale idéntica en los dos libros porque el fondo se calcula UNA vez. Publicar un único «CAPEX total» y pedir además el fondo en el otro libro es el error que hace que un mismo negocio aparezca con dos inversiones distintas en el mismo pack.</t>
         </is>
@@ -6531,8 +6552,8 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="3">
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A27:D27"/>
   </mergeCells>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>